<commit_message>
NPB自動更新(2軍): 2026-08-29 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/games/datamart/2026-08-29.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/games/datamart/2026-08-29.xlsx
@@ -107018,7 +107018,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>7回裏にレフトスタンドへ勝ち越しソロホームランを放ち、チームを勝利に導いた。</t>
+          <t>7回裏にレフトスタンドへ勝ち越しホームランを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -107043,7 +107043,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>7回表にライトへの逆転タイムリーヒットを放ち、試合の流れを大きく変えた。</t>
+          <t>7回表にランナー二三塁からライトへ逆転タイムリーヒットを放ち、試合の流れを変えた。</t>
         </is>
       </c>
     </row>
@@ -107068,7 +107068,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8回表にセンターへ勝ち越しタイムリーヒットを放ち、チームの勝利に貢献した。</t>
+          <t>8回表にランナー一二塁からセンターへ勝ち越しタイムリーヒットを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -107093,7 +107093,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>8回表にセンターへの勝ち越しタイムリーツーベースで、チームを優位に立たせた。</t>
+          <t>8回表にセンターへの勝ち越しタイムリーツーベースを放ち、試合の均衡を破った。</t>
         </is>
       </c>
     </row>
@@ -107118,7 +107118,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1回裏に先制3ランホームランを放ち、打線爆発の口火を切る活躍を見せた。</t>
+          <t>1回裏に先制3ランホームランを放ち、さらに猛打賞で4打点と大活躍した。</t>
         </is>
       </c>
     </row>
@@ -107143,7 +107143,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3回裏にレフトスタンドへ3ランホームランを放ち、チームのリードを大きく広げた。</t>
+          <t>3回裏にレフトスタンドへ3ランホームランを放ち、チームの大量リードに貢献した。</t>
         </is>
       </c>
     </row>

</xml_diff>